<commit_message>
Update CAIR integration with new provider organization handling and documentation improvements
- Modified .env.example to include PROVIDER_ORG_ID for clinic site organization.
- Updated CairSubmissionRepository and related models to utilize provider_org_id for submissions.
- Enhanced HL7 message builder to correctly map provider information and sanitize address fields.
- Added new scripts for inspecting and updating Excel mapping modifications.
- Improved CAIR Test Flow documentation to reflect recent changes and clarify endpoint usage.
- Introduced functionality for retrying submissions and resetting their status in the database.
</commit_message>
<xml_diff>
--- a/Required Fields mapping with DB 2-11-2021_Modified (2)_updated.xlsx
+++ b/Required Fields mapping with DB 2-11-2021_Modified (2)_updated.xlsx
@@ -743,6 +743,11 @@
           <t>Config</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED: vendor/integration org SF-013259 via .env SENDING_FACILITY_ID. Used in MSH-4, PID-3.4, ORC placer/filler, SOAP facilityID. Different from clinic site org in MSH-22.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -777,7 +782,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use CAIR2 per CAIR sample HL7 (not CAIRLO). Config: RECEIVING_FACILITY=CAIR2.</t>
+          <t>IMPLEMENTED: CAIR2 via .env RECEIVING_FACILITY (not CAIRLO).</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1011,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Confirmed: send AL (not ER). CAIR sample uses AL|AL.</t>
+          <t>IMPLEMENTED: send AL (not ER). CAIR sample uses AL|AL.</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1053,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Confirmed: send AL (not ER). CAIR sample uses AL|AL.</t>
+          <t>IMPLEMENTED: send AL. CAIR sample uses AL|AL.</t>
         </is>
       </c>
     </row>
@@ -1105,6 +1110,11 @@
           <t>DB (Facility ID)</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED: clinic site org from .env PROVIDER_ORG_ID=SF-012218 (tested OK on CAIR stage). Must match RXA-11.4. Do NOT use vendor SF-013259 — CAIR rejects vendor in MSH-22. Sample CA0054321 also rejected. Longer term: Locations.CairOrgCode from DB.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1178,7 +1188,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Use CAIR org code SF-013259 as assigning authority (CAIR sample: AC10293^^^CA0012345^MR). Not the EHR app name.</t>
+          <t>IMPLEMENTED: assigning authority = SENDING_FACILITY_ID (SF-013259). Not the EHR app name.</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1226,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Use MR per CAIR sample HL7 (Medical Record Number), not PI.</t>
+          <t>IMPLEMENTED: MR (Medical Record Number), not PI.</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1337,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Map ClaudMD GenderId: 1=M, 2=F, 3/Other=U. Implemented in worker.</t>
+          <t>IMPLEMENTED: GenderId map 1=M, 2=F, 3/Other=U in worker.</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1375,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Map to CDC CDCREC race code if Patients has race field; CAIR sample: 2106-3^^CDCREC. No race column mapped yet — EMR to confirm source.</t>
+          <t>IMPLEMENTED: Patients.RaceId -&gt; DataGroups.Description -&gt; CDCREC (cdc_codes.py). Example White=2106-3^^CDCREC (RaceId 1082). CAIR warns if empty — fill RaceId in DB.</t>
         </is>
       </c>
     </row>
@@ -1418,6 +1428,11 @@
         </is>
       </c>
       <c r="H23" s="29" t="n"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED: Patients.Address1/City/State/ZipCode when all set. Sanitize skips placeholders (ADDRESS 1*). CAIR rejects non-street values (e.g. GAMPAHA). Use a real street line or leave blank.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1445,7 +1460,7 @@
       <c r="H24" s="29" t="n"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>REQUIRED per CAIR email — at least one of home phone, cell, or email. DB: Patients.HomePhone, CellPhone, Email. Do not leave empty.</t>
+          <t>IMPLEMENTED: Patients.HomePhone, CellPhone, Email in PID-13 (PRN/PH, PRN/CP, NET/Internet). Required by CAIR email — do not leave empty.</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1523,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Map to CDC CDCREC ethnicity code if available; CAIR sample: 2186-5^^CDCREC. EMR to confirm source column.</t>
+          <t>IMPLEMENTED: Patients.EthnicityId -&gt; DataGroups.Description -&gt; CDCREC. Example Not Hispanic or Latino=2186-5^^CDCREC (EthnicityId 1084). CAIR warns if empty — fill EthnicityId in DB.</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1690,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>No DB column today. CAIR sample uses N (data can be shared). Y = lock from other providers. Default N unless EMR adds consent field.</t>
+          <t>IMPLEMENTED default N (shareable) per CAIR sample. No DB consent column yet. Y = lock from other providers.</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1728,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Use EHRVaccines.VaccineDate (or visit date) when PD1-12 has no DB source. CAIR sample: 20260810.</t>
+          <t>IMPLEMENTED: EHRVaccines.VaccineDate (or visit date) when PD1-12 sent.</t>
         </is>
       </c>
     </row>
@@ -1906,6 +1921,11 @@
         </is>
       </c>
       <c r="H40" s="29" t="n"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED: Providers.NationalProviderIdentifier + name via CheckInsHeader.ProviderId. XCN format: NPI^Last^First^^^^^^NPPES&amp;2.16.840.1.113883.4.6&amp;ISO^^^^NPI (component 9 HD assigning authority — CAIR ORC-12.9 warning cleared). OPEN: ORC-12.21 professional suffix (MD/NP/RN) not in DB/code yet — CAIR warning.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -2038,7 +2058,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Use EHRVaccines.VaccineDate + VaccineTime when set; else CheckInsHeader.CheckInDate + CheckInTime.</t>
+          <t>IMPLEMENTED: EHRVaccines.VaccineDate + VaccineTime when set; else CheckInsHeader.CheckInDate + CheckInTime.</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2100,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ClaudMD: ServiceCodes.NDCNumber (join via EHRVaccines.ServiceCodeId). CVX: add ServiceCodes.CvxCode (not in DB yet). CAIR accepts CVX or NDC, not both.</t>
+          <t>IMPLEMENTED: ServiceCodes.NDCNumber (via EHRVaccines.ServiceCodeId), dashed 11-digit form (e.g. 58160-0842-52^^NDC). CVX: ServiceCodes.CvxCode not in DB yet. CAIR accepts CVX or NDC, not both.</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2143,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ClaudMD: EHRVaccines.Dosage. If unknown send 999 with blank RXA-7 per CAIR rule.</t>
+          <t>IMPLEMENTED: EHRVaccines.Dosage. If unknown send 999 with blank RXA-7. CAIR may still return informational RXA-6 warning for some values.</t>
         </is>
       </c>
     </row>
@@ -2291,6 +2311,11 @@
           <t>DB (Facility ID)</t>
         </is>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED: same as MSH-22 — .env PROVIDER_ORG_ID=SF-012218 (^^^SF-012218). Required when RXA-9.1=00. Not vendor SF-013259.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -2331,7 +2356,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ClaudMD: EHRVaccines.LotNumber. Required when RXA-9=00.</t>
+          <t>IMPLEMENTED: EHRVaccines.LotNumber. Required when RXA-9=00.</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2551,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Confirmed: 1 per CAIR sample HL7.</t>
+          <t>IMPLEMENTED: two OBX segments — OBX-1 VFC eligibility (64994-7 / V01); OBX-2 funding source (30963-3 / PHC70^Private^CDCPHINVS).</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2709,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Confirmed: V01 (Not VFC eligible). Do not leave blank — CAIR sample uses V01.</t>
+          <t>IMPLEMENTED: V01 (Not VFC eligible). Do not leave blank.</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2808,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Confirmed: F (Final) per CAIR sample HL7.</t>
+          <t>IMPLEMENTED: F (Final).</t>
         </is>
       </c>
     </row>

</xml_diff>